<commit_message>
Update timelog and fix typo
</commit_message>
<xml_diff>
--- a/backend/backend-timelog.xlsx
+++ b/backend/backend-timelog.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="13">
   <si>
     <t xml:space="preserve">Total hours:</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t xml:space="preserve">Testien kirjottaminen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testien kirjottaminen ja koodin refaktorointi</t>
   </si>
 </sst>
 </file>
@@ -281,7 +284,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.78"/>
@@ -294,7 +297,7 @@
       </c>
       <c r="B1" s="2" t="n">
         <f aca="false">SUM(D:D)</f>
-        <v>1.32291666666667</v>
+        <v>1.46875</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -630,6 +633,27 @@
       </c>
       <c r="F18" s="1" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <f aca="false">C19-B19</f>
+        <v>0.145833333333333</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>